<commit_message>
Enhance scoring and processing logic in sensor pipeline
- Updated scoring functions in matcher.py to require at least one non-blank hardware identifier in SFM for Approach 1 and Approach 3.
- Modified process_batch method in orchestrator.py to introduce a delay between processing multiple sensor events to avoid rate limiting.
- Expanded demo event dataset in sensor_ingestor.py to include 35 realistic sensor events covering all service classifications and pipeline tiers, with detailed descriptions and timestamps.
- Implemented LLM verification for partial matches in service_classifier.py, allowing the model to confirm or adjust confidence in fuzzy matches, enhancing accuracy in service classification.

Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/data/test/test_ifm_demo.xlsx
+++ b/data/test/test_ifm_demo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="389">
   <si>
     <t>asset_id</t>
   </si>
@@ -160,6 +160,24 @@
     <t>IFM-025</t>
   </si>
   <si>
+    <t>IFM-A01</t>
+  </si>
+  <si>
+    <t>IFM-A02</t>
+  </si>
+  <si>
+    <t>IFM-A03</t>
+  </si>
+  <si>
+    <t>IFM-A04</t>
+  </si>
+  <si>
+    <t>IFM-A05</t>
+  </si>
+  <si>
+    <t>IFM-A06</t>
+  </si>
+  <si>
     <t>ALT-001</t>
   </si>
   <si>
@@ -259,6 +277,24 @@
     <t>ALT-025</t>
   </si>
   <si>
+    <t>ALTA-01</t>
+  </si>
+  <si>
+    <t>ALTA-02</t>
+  </si>
+  <si>
+    <t>ALTA-03</t>
+  </si>
+  <si>
+    <t>ALTA-04</t>
+  </si>
+  <si>
+    <t>ALTA-05</t>
+  </si>
+  <si>
+    <t>ALTA-06</t>
+  </si>
+  <si>
     <t>Boiler, Steam, Fire Tube(BLR-01A)</t>
   </si>
   <si>
@@ -358,6 +394,24 @@
     <t>Heat Exchanger(HX-LOOP-1)</t>
   </si>
   <si>
+    <t>Cooling System Controller(COOLING-CTRL-01)</t>
+  </si>
+  <si>
+    <t>Fan Coil Unit B2 Level 1(FCU-B2-L01)</t>
+  </si>
+  <si>
+    <t>Condenser Water Pump No. 2</t>
+  </si>
+  <si>
+    <t>Building Automation Controller 02</t>
+  </si>
+  <si>
+    <t>Emergency Backup Generator Unit Alpha</t>
+  </si>
+  <si>
+    <t>Commercial Water Chiller System B</t>
+  </si>
+  <si>
     <t>ACTIVE</t>
   </si>
   <si>
@@ -406,12 +460,6 @@
     <t>York</t>
   </si>
   <si>
-    <t>Taco</t>
-  </si>
-  <si>
-    <t>Ingersoll Rand</t>
-  </si>
-  <si>
     <t>Cummins</t>
   </si>
   <si>
@@ -580,6 +628,9 @@
     <t>M10-BFM</t>
   </si>
   <si>
+    <t>Desigo</t>
+  </si>
+  <si>
     <t>Boiler, Steam, Fire Tube</t>
   </si>
   <si>
@@ -664,6 +715,12 @@
     <t>Plate Heat Exchanger</t>
   </si>
   <si>
+    <t>BAS Controller</t>
+  </si>
+  <si>
+    <t>Chiller</t>
+  </si>
+  <si>
     <t>BLR-01A</t>
   </si>
   <si>
@@ -709,13 +766,13 @@
     <t>AHU-PH</t>
   </si>
   <si>
-    <t>HC-3</t>
+    <t>HTG-03</t>
   </si>
   <si>
     <t>SF-B2</t>
   </si>
   <si>
-    <t>CWP-Loop-1</t>
+    <t>COND-PMP-01</t>
   </si>
   <si>
     <t>EXH-RF-04</t>
@@ -763,12 +820,27 @@
     <t>HX-LOOP-1</t>
   </si>
   <si>
+    <t>COOLING-CTRL-01</t>
+  </si>
+  <si>
+    <t>FCU-B2-L01</t>
+  </si>
+  <si>
+    <t>PUMP-C-002</t>
+  </si>
+  <si>
+    <t>BAC-02</t>
+  </si>
+  <si>
+    <t>EBG-ALPHA</t>
+  </si>
+  <si>
+    <t>CWC-B</t>
+  </si>
+  <si>
     <t>Boiler</t>
   </si>
   <si>
-    <t>Chiller</t>
-  </si>
-  <si>
     <t>Pump</t>
   </si>
   <si>
@@ -877,6 +949,15 @@
     <t>US, MA, Boston</t>
   </si>
   <si>
+    <t>US, GA, Savannah</t>
+  </si>
+  <si>
+    <t>US, PA, Pittsburgh</t>
+  </si>
+  <si>
+    <t>US, AZ, Tucson</t>
+  </si>
+  <si>
     <t>Pleasanton Campus - Building A</t>
   </si>
   <si>
@@ -967,6 +1048,24 @@
     <t>Boston Innovation Center</t>
   </si>
   <si>
+    <t>Savannah Operations Center</t>
+  </si>
+  <si>
+    <t>Minneapolis North Tower</t>
+  </si>
+  <si>
+    <t>Milwaukee Central Utility Plant</t>
+  </si>
+  <si>
+    <t>Pittsburgh Campus East Wing</t>
+  </si>
+  <si>
+    <t>Tucson Data Hub</t>
+  </si>
+  <si>
+    <t>Charlotte Cooling Plant</t>
+  </si>
+  <si>
     <t>Roof</t>
   </si>
   <si>
@@ -1012,6 +1111,9 @@
     <t>Level B2</t>
   </si>
   <si>
+    <t>Level 2</t>
+  </si>
+  <si>
     <t>Mechanical</t>
   </si>
   <si>
@@ -1067,6 +1169,15 @@
   </si>
   <si>
     <t>Electrical Room</t>
+  </si>
+  <si>
+    <t>Control Room</t>
+  </si>
+  <si>
+    <t>Room 101</t>
+  </si>
+  <si>
+    <t>Chiller Plant</t>
   </si>
   <si>
     <t>Clorox</t>
@@ -1427,7 +1538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O34"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:15">
@@ -1482,46 +1593,46 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="D2" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E2" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
       <c r="F2" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
       <c r="G2" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="H2" t="s">
-        <v>188</v>
+        <v>205</v>
       </c>
       <c r="I2" t="s">
-        <v>216</v>
+        <v>235</v>
       </c>
       <c r="J2" t="s">
-        <v>249</v>
+        <v>274</v>
       </c>
       <c r="K2" t="s">
-        <v>261</v>
+        <v>285</v>
       </c>
       <c r="L2" t="s">
-        <v>287</v>
+        <v>314</v>
       </c>
       <c r="M2" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
       <c r="N2" t="s">
-        <v>332</v>
+        <v>366</v>
       </c>
       <c r="O2" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -1529,46 +1640,46 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="D3" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E3" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="F3" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="G3" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="H3" t="s">
-        <v>189</v>
+        <v>206</v>
       </c>
       <c r="I3" t="s">
-        <v>217</v>
+        <v>236</v>
       </c>
       <c r="J3" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="K3" t="s">
-        <v>261</v>
+        <v>285</v>
       </c>
       <c r="L3" t="s">
-        <v>288</v>
+        <v>315</v>
       </c>
       <c r="M3" t="s">
-        <v>318</v>
+        <v>351</v>
       </c>
       <c r="N3" t="s">
-        <v>333</v>
+        <v>367</v>
       </c>
       <c r="O3" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -1576,46 +1687,46 @@
         <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E4" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="F4" t="s">
-        <v>144</v>
+        <v>160</v>
       </c>
       <c r="G4" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="H4" t="s">
-        <v>190</v>
+        <v>207</v>
       </c>
       <c r="I4" t="s">
-        <v>218</v>
+        <v>237</v>
       </c>
       <c r="J4" t="s">
-        <v>250</v>
+        <v>234</v>
       </c>
       <c r="K4" t="s">
-        <v>262</v>
+        <v>286</v>
       </c>
       <c r="L4" t="s">
-        <v>289</v>
+        <v>316</v>
       </c>
       <c r="M4" t="s">
-        <v>319</v>
+        <v>352</v>
       </c>
       <c r="N4" t="s">
-        <v>334</v>
+        <v>368</v>
       </c>
       <c r="O4" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -1623,46 +1734,46 @@
         <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D5" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E5" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="F5" t="s">
-        <v>145</v>
+        <v>161</v>
       </c>
       <c r="G5" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="H5" t="s">
-        <v>191</v>
+        <v>208</v>
       </c>
       <c r="I5" t="s">
-        <v>219</v>
+        <v>238</v>
       </c>
       <c r="J5" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="K5" t="s">
-        <v>261</v>
+        <v>285</v>
       </c>
       <c r="L5" t="s">
-        <v>287</v>
+        <v>314</v>
       </c>
       <c r="M5" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
       <c r="N5" t="s">
-        <v>335</v>
+        <v>369</v>
       </c>
       <c r="O5" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -1670,46 +1781,46 @@
         <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="D6" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E6" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
       <c r="F6" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
       <c r="G6" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="H6" t="s">
-        <v>192</v>
+        <v>209</v>
       </c>
       <c r="I6" t="s">
-        <v>220</v>
+        <v>239</v>
       </c>
       <c r="J6" t="s">
-        <v>251</v>
+        <v>275</v>
       </c>
       <c r="K6" t="s">
-        <v>263</v>
+        <v>287</v>
       </c>
       <c r="L6" t="s">
-        <v>290</v>
+        <v>317</v>
       </c>
       <c r="M6" t="s">
-        <v>320</v>
+        <v>353</v>
       </c>
       <c r="N6" t="s">
-        <v>336</v>
+        <v>370</v>
       </c>
       <c r="O6" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -1717,46 +1828,46 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C7" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="D7" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E7" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="F7" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="G7" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="H7" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="I7" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
       <c r="J7" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="K7" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
       <c r="L7" t="s">
-        <v>291</v>
+        <v>318</v>
       </c>
       <c r="M7" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
       <c r="N7" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
       <c r="O7" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -1764,46 +1875,46 @@
         <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="C8" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="D8" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E8" t="s">
-        <v>123</v>
+        <v>141</v>
       </c>
       <c r="F8" t="s">
-        <v>148</v>
+        <v>164</v>
       </c>
       <c r="G8" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
       <c r="H8" t="s">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="I8" t="s">
-        <v>222</v>
+        <v>241</v>
       </c>
       <c r="J8" t="s">
-        <v>252</v>
+        <v>276</v>
       </c>
       <c r="K8" t="s">
-        <v>265</v>
+        <v>289</v>
       </c>
       <c r="L8" t="s">
-        <v>292</v>
+        <v>319</v>
       </c>
       <c r="M8" t="s">
-        <v>321</v>
+        <v>354</v>
       </c>
       <c r="N8" t="s">
-        <v>337</v>
+        <v>371</v>
       </c>
       <c r="O8" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -1811,46 +1922,46 @@
         <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C9" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="D9" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E9" t="s">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="F9" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="G9" t="s">
-        <v>172</v>
+        <v>188</v>
       </c>
       <c r="H9" t="s">
-        <v>195</v>
+        <v>212</v>
       </c>
       <c r="I9" t="s">
-        <v>223</v>
+        <v>242</v>
       </c>
       <c r="J9" t="s">
-        <v>195</v>
+        <v>212</v>
       </c>
       <c r="K9" t="s">
-        <v>266</v>
+        <v>290</v>
       </c>
       <c r="L9" t="s">
-        <v>293</v>
+        <v>320</v>
       </c>
       <c r="M9" t="s">
-        <v>319</v>
+        <v>352</v>
       </c>
       <c r="N9" t="s">
-        <v>334</v>
+        <v>368</v>
       </c>
       <c r="O9" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -1858,46 +1969,46 @@
         <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C10" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="D10" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E10" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="F10" t="s">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="G10" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="H10" t="s">
-        <v>196</v>
+        <v>213</v>
       </c>
       <c r="I10" t="s">
-        <v>224</v>
+        <v>243</v>
       </c>
       <c r="J10" t="s">
-        <v>196</v>
+        <v>213</v>
       </c>
       <c r="K10" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="L10" t="s">
-        <v>294</v>
+        <v>321</v>
       </c>
       <c r="M10" t="s">
-        <v>322</v>
+        <v>355</v>
       </c>
       <c r="N10" t="s">
-        <v>338</v>
+        <v>372</v>
       </c>
       <c r="O10" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -1905,46 +2016,46 @@
         <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="C11" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="D11" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E11" t="s">
-        <v>126</v>
+        <v>144</v>
       </c>
       <c r="F11" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="G11" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="H11" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="I11" t="s">
-        <v>225</v>
+        <v>244</v>
       </c>
       <c r="J11" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="K11" t="s">
-        <v>268</v>
+        <v>292</v>
       </c>
       <c r="L11" t="s">
-        <v>295</v>
+        <v>322</v>
       </c>
       <c r="M11" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
       <c r="N11" t="s">
-        <v>339</v>
+        <v>373</v>
       </c>
       <c r="O11" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -1952,46 +2063,46 @@
         <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D12" t="s">
-        <v>115</v>
+        <v>133</v>
       </c>
       <c r="E12" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="F12" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="G12" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="H12" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="I12" t="s">
-        <v>226</v>
+        <v>245</v>
       </c>
       <c r="J12" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="K12" t="s">
-        <v>261</v>
+        <v>285</v>
       </c>
       <c r="L12" t="s">
-        <v>288</v>
+        <v>315</v>
       </c>
       <c r="M12" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
       <c r="N12" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
       <c r="O12" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -1999,37 +2110,37 @@
         <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C13" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="D13" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="H13" t="s">
-        <v>199</v>
+        <v>216</v>
       </c>
       <c r="I13" t="s">
-        <v>227</v>
+        <v>246</v>
       </c>
       <c r="J13" t="s">
-        <v>251</v>
+        <v>275</v>
       </c>
       <c r="K13" t="s">
-        <v>266</v>
+        <v>290</v>
       </c>
       <c r="L13" t="s">
-        <v>296</v>
+        <v>323</v>
       </c>
       <c r="M13" t="s">
-        <v>320</v>
+        <v>353</v>
       </c>
       <c r="N13" t="s">
-        <v>336</v>
+        <v>370</v>
       </c>
       <c r="O13" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -2037,46 +2148,46 @@
         <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C14" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="D14" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E14" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="F14" t="s">
-        <v>153</v>
+        <v>169</v>
       </c>
       <c r="G14" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
       <c r="H14" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="I14" t="s">
-        <v>228</v>
+        <v>247</v>
       </c>
       <c r="J14" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="K14" t="s">
-        <v>269</v>
+        <v>293</v>
       </c>
       <c r="L14" t="s">
-        <v>297</v>
+        <v>324</v>
       </c>
       <c r="M14" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
       <c r="N14" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
       <c r="O14" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="15" spans="1:15">
@@ -2084,43 +2195,43 @@
         <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C15" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="D15" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E15" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="G15" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="H15" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="I15" t="s">
-        <v>229</v>
+        <v>248</v>
       </c>
       <c r="J15" t="s">
-        <v>252</v>
+        <v>276</v>
       </c>
       <c r="K15" t="s">
-        <v>270</v>
+        <v>294</v>
       </c>
       <c r="L15" t="s">
-        <v>298</v>
+        <v>325</v>
       </c>
       <c r="M15" t="s">
-        <v>323</v>
+        <v>356</v>
       </c>
       <c r="N15" t="s">
-        <v>340</v>
+        <v>374</v>
       </c>
       <c r="O15" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="16" spans="1:15">
@@ -2128,46 +2239,46 @@
         <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C16" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="D16" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E16" t="s">
-        <v>129</v>
+        <v>147</v>
       </c>
       <c r="F16" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="G16" t="s">
-        <v>177</v>
+        <v>193</v>
       </c>
       <c r="H16" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="I16" t="s">
-        <v>230</v>
+        <v>249</v>
       </c>
       <c r="J16" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="K16" t="s">
-        <v>271</v>
+        <v>295</v>
       </c>
       <c r="L16" t="s">
-        <v>299</v>
+        <v>326</v>
       </c>
       <c r="M16" t="s">
-        <v>324</v>
+        <v>357</v>
       </c>
       <c r="N16" t="s">
-        <v>332</v>
+        <v>366</v>
       </c>
       <c r="O16" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -2175,37 +2286,37 @@
         <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="C17" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="D17" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="H17" t="s">
-        <v>202</v>
+        <v>219</v>
       </c>
       <c r="I17" t="s">
-        <v>231</v>
+        <v>250</v>
       </c>
       <c r="J17" t="s">
-        <v>253</v>
+        <v>277</v>
       </c>
       <c r="K17" t="s">
-        <v>272</v>
+        <v>296</v>
       </c>
       <c r="L17" t="s">
-        <v>300</v>
+        <v>327</v>
       </c>
       <c r="M17" t="s">
-        <v>325</v>
+        <v>358</v>
       </c>
       <c r="N17" t="s">
-        <v>332</v>
+        <v>366</v>
       </c>
       <c r="O17" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="18" spans="1:15">
@@ -2213,37 +2324,37 @@
         <v>31</v>
       </c>
       <c r="B18" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C18" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="D18" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="H18" t="s">
-        <v>203</v>
+        <v>220</v>
       </c>
       <c r="I18" t="s">
-        <v>232</v>
+        <v>251</v>
       </c>
       <c r="J18" t="s">
-        <v>203</v>
+        <v>220</v>
       </c>
       <c r="K18" t="s">
-        <v>273</v>
+        <v>297</v>
       </c>
       <c r="L18" t="s">
-        <v>301</v>
+        <v>328</v>
       </c>
       <c r="M18" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
       <c r="N18" t="s">
-        <v>341</v>
+        <v>375</v>
       </c>
       <c r="O18" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="19" spans="1:15">
@@ -2251,40 +2362,37 @@
         <v>32</v>
       </c>
       <c r="B19" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="C19" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="D19" t="s">
-        <v>114</v>
-      </c>
-      <c r="E19" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H19" t="s">
-        <v>204</v>
+        <v>221</v>
       </c>
       <c r="I19" t="s">
-        <v>233</v>
+        <v>252</v>
       </c>
       <c r="J19" t="s">
-        <v>251</v>
+        <v>275</v>
       </c>
       <c r="K19" t="s">
-        <v>274</v>
+        <v>298</v>
       </c>
       <c r="L19" t="s">
-        <v>302</v>
+        <v>329</v>
       </c>
       <c r="M19" t="s">
-        <v>320</v>
+        <v>353</v>
       </c>
       <c r="N19" t="s">
-        <v>336</v>
+        <v>370</v>
       </c>
       <c r="O19" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="20" spans="1:15">
@@ -2292,37 +2400,37 @@
         <v>33</v>
       </c>
       <c r="B20" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C20" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="D20" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="H20" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="I20" t="s">
-        <v>234</v>
+        <v>253</v>
       </c>
       <c r="J20" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="K20" t="s">
-        <v>275</v>
+        <v>299</v>
       </c>
       <c r="L20" t="s">
-        <v>303</v>
+        <v>330</v>
       </c>
       <c r="M20" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
       <c r="N20" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
       <c r="O20" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="21" spans="1:15">
@@ -2330,40 +2438,37 @@
         <v>34</v>
       </c>
       <c r="B21" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C21" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="D21" t="s">
-        <v>114</v>
-      </c>
-      <c r="E21" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H21" t="s">
-        <v>205</v>
+        <v>222</v>
       </c>
       <c r="I21" t="s">
-        <v>235</v>
+        <v>254</v>
       </c>
       <c r="J21" t="s">
-        <v>205</v>
+        <v>222</v>
       </c>
       <c r="K21" t="s">
-        <v>276</v>
+        <v>300</v>
       </c>
       <c r="L21" t="s">
-        <v>304</v>
+        <v>331</v>
       </c>
       <c r="M21" t="s">
-        <v>326</v>
+        <v>359</v>
       </c>
       <c r="N21" t="s">
-        <v>342</v>
+        <v>376</v>
       </c>
       <c r="O21" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -2371,37 +2476,37 @@
         <v>35</v>
       </c>
       <c r="B22" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C22" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="D22" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="H22" t="s">
-        <v>206</v>
+        <v>223</v>
       </c>
       <c r="I22" t="s">
-        <v>236</v>
+        <v>255</v>
       </c>
       <c r="J22" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="K22" t="s">
-        <v>277</v>
+        <v>301</v>
       </c>
       <c r="L22" t="s">
-        <v>305</v>
+        <v>332</v>
       </c>
       <c r="M22" t="s">
-        <v>327</v>
+        <v>360</v>
       </c>
       <c r="N22" t="s">
-        <v>332</v>
+        <v>366</v>
       </c>
       <c r="O22" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="23" spans="1:15">
@@ -2409,37 +2514,37 @@
         <v>36</v>
       </c>
       <c r="B23" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C23" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="D23" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="H23" t="s">
-        <v>207</v>
+        <v>224</v>
       </c>
       <c r="I23" t="s">
-        <v>237</v>
+        <v>256</v>
       </c>
       <c r="J23" t="s">
-        <v>254</v>
+        <v>278</v>
       </c>
       <c r="K23" t="s">
-        <v>278</v>
+        <v>302</v>
       </c>
       <c r="L23" t="s">
-        <v>306</v>
+        <v>333</v>
       </c>
       <c r="M23" t="s">
-        <v>320</v>
+        <v>353</v>
       </c>
       <c r="N23" t="s">
-        <v>343</v>
+        <v>377</v>
       </c>
       <c r="O23" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="24" spans="1:15">
@@ -2447,37 +2552,37 @@
         <v>37</v>
       </c>
       <c r="B24" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C24" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="D24" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="H24" t="s">
-        <v>208</v>
+        <v>225</v>
       </c>
       <c r="I24" t="s">
-        <v>238</v>
+        <v>257</v>
       </c>
       <c r="J24" t="s">
-        <v>255</v>
+        <v>279</v>
       </c>
       <c r="K24" t="s">
-        <v>279</v>
+        <v>303</v>
       </c>
       <c r="L24" t="s">
-        <v>307</v>
+        <v>334</v>
       </c>
       <c r="M24" t="s">
-        <v>328</v>
+        <v>361</v>
       </c>
       <c r="N24" t="s">
-        <v>344</v>
+        <v>378</v>
       </c>
       <c r="O24" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="25" spans="1:15">
@@ -2485,46 +2590,46 @@
         <v>38</v>
       </c>
       <c r="B25" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C25" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="D25" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E25" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="F25" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="G25" t="s">
-        <v>178</v>
+        <v>194</v>
       </c>
       <c r="H25" t="s">
-        <v>208</v>
+        <v>225</v>
       </c>
       <c r="I25" t="s">
-        <v>239</v>
+        <v>258</v>
       </c>
       <c r="J25" t="s">
-        <v>255</v>
+        <v>279</v>
       </c>
       <c r="K25" t="s">
-        <v>280</v>
+        <v>304</v>
       </c>
       <c r="L25" t="s">
-        <v>308</v>
+        <v>335</v>
       </c>
       <c r="M25" t="s">
-        <v>328</v>
+        <v>361</v>
       </c>
       <c r="N25" t="s">
-        <v>345</v>
+        <v>379</v>
       </c>
       <c r="O25" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="26" spans="1:15">
@@ -2532,46 +2637,46 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="C26" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="D26" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E26" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="F26" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="G26" t="s">
-        <v>179</v>
+        <v>195</v>
       </c>
       <c r="H26" t="s">
-        <v>209</v>
+        <v>226</v>
       </c>
       <c r="I26" t="s">
-        <v>240</v>
+        <v>259</v>
       </c>
       <c r="J26" t="s">
-        <v>209</v>
+        <v>226</v>
       </c>
       <c r="K26" t="s">
-        <v>281</v>
+        <v>305</v>
       </c>
       <c r="L26" t="s">
-        <v>309</v>
+        <v>336</v>
       </c>
       <c r="M26" t="s">
-        <v>329</v>
+        <v>362</v>
       </c>
       <c r="N26" t="s">
-        <v>346</v>
+        <v>380</v>
       </c>
       <c r="O26" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="27" spans="1:15">
@@ -2579,46 +2684,46 @@
         <v>40</v>
       </c>
       <c r="B27" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C27" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="D27" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E27" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F27" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="G27" t="s">
-        <v>180</v>
+        <v>196</v>
       </c>
       <c r="H27" t="s">
-        <v>210</v>
+        <v>227</v>
       </c>
       <c r="I27" t="s">
-        <v>241</v>
+        <v>260</v>
       </c>
       <c r="J27" t="s">
-        <v>256</v>
+        <v>280</v>
       </c>
       <c r="K27" t="s">
-        <v>272</v>
+        <v>296</v>
       </c>
       <c r="L27" t="s">
-        <v>310</v>
+        <v>337</v>
       </c>
       <c r="M27" t="s">
-        <v>330</v>
+        <v>363</v>
       </c>
       <c r="N27" t="s">
-        <v>347</v>
+        <v>381</v>
       </c>
       <c r="O27" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="28" spans="1:15">
@@ -2626,46 +2731,46 @@
         <v>41</v>
       </c>
       <c r="B28" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="C28" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D28" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E28" t="s">
-        <v>135</v>
+        <v>151</v>
       </c>
       <c r="F28" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="G28" t="s">
-        <v>181</v>
+        <v>197</v>
       </c>
       <c r="H28" t="s">
-        <v>211</v>
+        <v>228</v>
       </c>
       <c r="I28" t="s">
-        <v>242</v>
+        <v>261</v>
       </c>
       <c r="J28" t="s">
-        <v>257</v>
+        <v>281</v>
       </c>
       <c r="K28" t="s">
-        <v>280</v>
+        <v>304</v>
       </c>
       <c r="L28" t="s">
-        <v>308</v>
+        <v>335</v>
       </c>
       <c r="M28" t="s">
-        <v>318</v>
+        <v>351</v>
       </c>
       <c r="N28" t="s">
-        <v>348</v>
+        <v>382</v>
       </c>
       <c r="O28" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="29" spans="1:15">
@@ -2673,46 +2778,46 @@
         <v>42</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="C29" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="D29" t="s">
-        <v>116</v>
+        <v>134</v>
       </c>
       <c r="E29" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="F29" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="G29" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="H29" t="s">
-        <v>205</v>
+        <v>222</v>
       </c>
       <c r="I29" t="s">
-        <v>243</v>
+        <v>262</v>
       </c>
       <c r="J29" t="s">
-        <v>205</v>
+        <v>222</v>
       </c>
       <c r="K29" t="s">
-        <v>282</v>
+        <v>306</v>
       </c>
       <c r="L29" t="s">
-        <v>311</v>
+        <v>338</v>
       </c>
       <c r="M29" t="s">
-        <v>326</v>
+        <v>359</v>
       </c>
       <c r="N29" t="s">
-        <v>342</v>
+        <v>376</v>
       </c>
       <c r="O29" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="30" spans="1:15">
@@ -2720,46 +2825,46 @@
         <v>43</v>
       </c>
       <c r="B30" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C30" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="D30" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E30" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
       <c r="F30" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="G30" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
       <c r="H30" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="I30" t="s">
-        <v>244</v>
+        <v>263</v>
       </c>
       <c r="J30" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="K30" t="s">
-        <v>283</v>
+        <v>307</v>
       </c>
       <c r="L30" t="s">
-        <v>312</v>
+        <v>339</v>
       </c>
       <c r="M30" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
       <c r="N30" t="s">
-        <v>341</v>
+        <v>375</v>
       </c>
       <c r="O30" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="31" spans="1:15">
@@ -2767,46 +2872,46 @@
         <v>44</v>
       </c>
       <c r="B31" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C31" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="D31" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E31" t="s">
-        <v>138</v>
+        <v>154</v>
       </c>
       <c r="F31" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="G31" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="H31" t="s">
-        <v>212</v>
+        <v>229</v>
       </c>
       <c r="I31" t="s">
-        <v>245</v>
+        <v>264</v>
       </c>
       <c r="J31" t="s">
-        <v>249</v>
+        <v>274</v>
       </c>
       <c r="K31" t="s">
-        <v>284</v>
+        <v>308</v>
       </c>
       <c r="L31" t="s">
-        <v>313</v>
+        <v>340</v>
       </c>
       <c r="M31" t="s">
-        <v>319</v>
+        <v>352</v>
       </c>
       <c r="N31" t="s">
-        <v>349</v>
+        <v>383</v>
       </c>
       <c r="O31" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="32" spans="1:15">
@@ -2814,46 +2919,46 @@
         <v>45</v>
       </c>
       <c r="B32" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C32" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="D32" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E32" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="F32" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="G32" t="s">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="H32" t="s">
-        <v>213</v>
+        <v>230</v>
       </c>
       <c r="I32" t="s">
-        <v>246</v>
+        <v>265</v>
       </c>
       <c r="J32" t="s">
-        <v>258</v>
+        <v>282</v>
       </c>
       <c r="K32" t="s">
-        <v>273</v>
+        <v>297</v>
       </c>
       <c r="L32" t="s">
-        <v>314</v>
+        <v>341</v>
       </c>
       <c r="M32" t="s">
-        <v>328</v>
+        <v>361</v>
       </c>
       <c r="N32" t="s">
-        <v>350</v>
+        <v>384</v>
       </c>
       <c r="O32" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="33" spans="1:15">
@@ -2861,46 +2966,46 @@
         <v>46</v>
       </c>
       <c r="B33" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="C33" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="D33" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E33" t="s">
-        <v>140</v>
+        <v>156</v>
       </c>
       <c r="F33" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
       <c r="G33" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="H33" t="s">
-        <v>214</v>
+        <v>231</v>
       </c>
       <c r="I33" t="s">
-        <v>247</v>
+        <v>266</v>
       </c>
       <c r="J33" t="s">
-        <v>259</v>
+        <v>283</v>
       </c>
       <c r="K33" t="s">
-        <v>285</v>
+        <v>309</v>
       </c>
       <c r="L33" t="s">
-        <v>315</v>
+        <v>342</v>
       </c>
       <c r="M33" t="s">
-        <v>322</v>
+        <v>355</v>
       </c>
       <c r="N33" t="s">
-        <v>348</v>
+        <v>382</v>
       </c>
       <c r="O33" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
     </row>
     <row r="34" spans="1:15">
@@ -2908,46 +3013,280 @@
         <v>47</v>
       </c>
       <c r="B34" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C34" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="D34" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="E34" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="F34" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="G34" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
       <c r="H34" t="s">
-        <v>215</v>
+        <v>232</v>
       </c>
       <c r="I34" t="s">
-        <v>248</v>
+        <v>267</v>
       </c>
       <c r="J34" t="s">
-        <v>260</v>
+        <v>284</v>
       </c>
       <c r="K34" t="s">
-        <v>286</v>
+        <v>310</v>
       </c>
       <c r="L34" t="s">
-        <v>316</v>
+        <v>343</v>
       </c>
       <c r="M34" t="s">
-        <v>331</v>
+        <v>364</v>
       </c>
       <c r="N34" t="s">
-        <v>333</v>
+        <v>367</v>
       </c>
       <c r="O34" t="s">
-        <v>351</v>
+        <v>388</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15">
+      <c r="A35" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35" t="s">
+        <v>87</v>
+      </c>
+      <c r="C35" t="s">
+        <v>126</v>
+      </c>
+      <c r="D35" t="s">
+        <v>132</v>
+      </c>
+      <c r="H35" t="s">
+        <v>233</v>
+      </c>
+      <c r="I35" t="s">
+        <v>268</v>
+      </c>
+      <c r="J35" t="s">
+        <v>233</v>
+      </c>
+      <c r="K35" t="s">
+        <v>311</v>
+      </c>
+      <c r="L35" t="s">
+        <v>344</v>
+      </c>
+      <c r="M35" t="s">
+        <v>365</v>
+      </c>
+      <c r="N35" t="s">
+        <v>385</v>
+      </c>
+      <c r="O35" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15">
+      <c r="A36" t="s">
+        <v>49</v>
+      </c>
+      <c r="B36" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" t="s">
+        <v>127</v>
+      </c>
+      <c r="D36" t="s">
+        <v>132</v>
+      </c>
+      <c r="H36" t="s">
+        <v>213</v>
+      </c>
+      <c r="I36" t="s">
+        <v>269</v>
+      </c>
+      <c r="J36" t="s">
+        <v>213</v>
+      </c>
+      <c r="K36" t="s">
+        <v>308</v>
+      </c>
+      <c r="L36" t="s">
+        <v>345</v>
+      </c>
+      <c r="M36" t="s">
+        <v>364</v>
+      </c>
+      <c r="N36" t="s">
+        <v>386</v>
+      </c>
+      <c r="O36" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15">
+      <c r="A37" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" t="s">
+        <v>89</v>
+      </c>
+      <c r="C37" t="s">
+        <v>128</v>
+      </c>
+      <c r="D37" t="s">
+        <v>132</v>
+      </c>
+      <c r="H37" t="s">
+        <v>221</v>
+      </c>
+      <c r="I37" t="s">
+        <v>270</v>
+      </c>
+      <c r="J37" t="s">
+        <v>275</v>
+      </c>
+      <c r="K37" t="s">
+        <v>306</v>
+      </c>
+      <c r="L37" t="s">
+        <v>346</v>
+      </c>
+      <c r="M37" t="s">
+        <v>353</v>
+      </c>
+      <c r="N37" t="s">
+        <v>370</v>
+      </c>
+      <c r="O37" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15">
+      <c r="A38" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" t="s">
+        <v>90</v>
+      </c>
+      <c r="C38" t="s">
+        <v>129</v>
+      </c>
+      <c r="D38" t="s">
+        <v>132</v>
+      </c>
+      <c r="E38" t="s">
+        <v>146</v>
+      </c>
+      <c r="G38" t="s">
+        <v>204</v>
+      </c>
+      <c r="H38" t="s">
+        <v>233</v>
+      </c>
+      <c r="I38" t="s">
+        <v>271</v>
+      </c>
+      <c r="J38" t="s">
+        <v>233</v>
+      </c>
+      <c r="K38" t="s">
+        <v>312</v>
+      </c>
+      <c r="L38" t="s">
+        <v>347</v>
+      </c>
+      <c r="M38" t="s">
+        <v>359</v>
+      </c>
+      <c r="N38" t="s">
+        <v>367</v>
+      </c>
+      <c r="O38" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15">
+      <c r="A39" t="s">
+        <v>52</v>
+      </c>
+      <c r="B39" t="s">
+        <v>91</v>
+      </c>
+      <c r="C39" t="s">
+        <v>130</v>
+      </c>
+      <c r="D39" t="s">
+        <v>132</v>
+      </c>
+      <c r="H39" t="s">
+        <v>225</v>
+      </c>
+      <c r="I39" t="s">
+        <v>272</v>
+      </c>
+      <c r="J39" t="s">
+        <v>279</v>
+      </c>
+      <c r="K39" t="s">
+        <v>313</v>
+      </c>
+      <c r="L39" t="s">
+        <v>348</v>
+      </c>
+      <c r="M39" t="s">
+        <v>361</v>
+      </c>
+      <c r="N39" t="s">
+        <v>378</v>
+      </c>
+      <c r="O39" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15">
+      <c r="A40" t="s">
+        <v>53</v>
+      </c>
+      <c r="B40" t="s">
+        <v>92</v>
+      </c>
+      <c r="C40" t="s">
+        <v>131</v>
+      </c>
+      <c r="D40" t="s">
+        <v>132</v>
+      </c>
+      <c r="H40" t="s">
+        <v>234</v>
+      </c>
+      <c r="I40" t="s">
+        <v>273</v>
+      </c>
+      <c r="J40" t="s">
+        <v>234</v>
+      </c>
+      <c r="K40" t="s">
+        <v>307</v>
+      </c>
+      <c r="L40" t="s">
+        <v>349</v>
+      </c>
+      <c r="M40" t="s">
+        <v>353</v>
+      </c>
+      <c r="N40" t="s">
+        <v>387</v>
+      </c>
+      <c r="O40" t="s">
+        <v>388</v>
       </c>
     </row>
   </sheetData>

</xml_diff>